<commit_message>
feat(backup): resolve backup dir and live db path commands
</commit_message>
<xml_diff>
--- a/docs/public/inventory - TEMPLATE.xlsx
+++ b/docs/public/inventory - TEMPLATE.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory Template" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory Template'!$A$1:$AO$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory Template'!$A$1:$AQ$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Inventory Template'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -455,7 +455,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AO101"/>
+  <dimension ref="A1:AQ101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -499,6 +499,8 @@
     <col width="16" customWidth="1" min="39" max="39"/>
     <col width="18" customWidth="1" min="40" max="40"/>
     <col width="20" customWidth="1" min="41" max="41"/>
+    <col width="12" customWidth="1" min="42" max="42"/>
+    <col width="12" customWidth="1" min="43" max="43"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -705,6 +707,16 @@
       <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>supplier</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>pack_qty</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>pack_unit</t>
         </is>
       </c>
     </row>
@@ -4909,7 +4921,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AO1"/>
+  <autoFilter ref="A1:AQ1"/>
   <conditionalFormatting sqref="F2:F501">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>10000</formula>
@@ -4926,16 +4938,16 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="9">
-    <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid strength" error="Strength must be 0–10000 or blank" promptTitle="Strength" prompt="Parts of the old DOSAGE — e.g. 500 + mg + tablet + 100/box" type="decimal" operator="between">
+  <dataValidations count="11">
+    <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid strength" error="Strength must be 20 characters or fewer" promptTitle="Strength" prompt="Parts of the old DOSAGE — e.g. 500 + mg + tablet + 100/box" type="textLength" operator="between">
       <formula1>0</formula1>
-      <formula2>10000</formula2>
+      <formula2>20</formula2>
     </dataValidation>
     <dataValidation sqref="C2:C501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid unit" error="Pick a unit or leave blank" promptTitle="Strength unit" prompt="Parts of the old DOSAGE — e.g. 500 + mg + tablet + 100/box" type="list">
       <formula1>"mg,g,mcg,ml,mg/ml,mg/5ml,%,IU,units"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid form" error="Pick a form or leave blank" promptTitle="Form" prompt="Parts of the old DOSAGE — e.g. 500 + mg + tablet + 100/box" type="list">
-      <formula1>"tablet,capsule,cap,sachet,syrup,suspension,susp,ointment,cream,drops,vial,ampule,nebule,injection,suppository,box,piece"</formula1>
+      <formula1>"tablet,capsule,cap,sachet,syrup,suspension,susp,ointment,cream,drops,vial,ampule,nebule,injection,suppository,box,piece,tabs,tab,inhaler,solution,gel,lotion,spray"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="textLength" operator="between">
       <formula1>0</formula1>
@@ -4960,6 +4972,14 @@
       <formula1>0</formula1>
       <formula2>80</formula2>
     </dataValidation>
+    <dataValidation sqref="AP2:AP501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid pack qty" error="Pack qty must be 0–10000" promptTitle="Pack qty" prompt="Units per pack, e.g. 100. Blank when unpacked." type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>10000</formula2>
+    </dataValidation>
+    <dataValidation sqref="AQ2:AQ501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" promptTitle="Pack unit" prompt="Pack unit, e.g. box. Blank when unpacked." type="textLength" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
+    </dataValidation>
   </dataValidations>
   <printOptions gridLines="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>